<commit_message>
fix: set TestScenario output path in Scenarios.xlsx
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Scenarios.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub repositories\ESQlabs\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\update-aciclovir-pkml\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F437A9AB-9A78-41D6-A0BE-980446BE39C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C66A711-427E-4337-901B-6EC532D0324A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="21840" windowHeight="37920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="690" yWindow="1450" windowWidth="27640" windowHeight="19270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="8" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="37">
   <si>
     <t>SimulationTime</t>
   </si>
@@ -522,24 +522,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A1BACA-04A5-4461-B34D-CB73BA82CEC5}">
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.140625" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7265625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -580,7 +580,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -602,8 +602,11 @@
       <c r="L2" t="s">
         <v>13</v>
       </c>
+      <c r="M2" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -638,7 +641,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -670,7 +673,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -702,7 +705,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -735,13 +738,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAA486CF-725F-421A-8D45-E3AE92A4A2C0}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -749,7 +752,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -757,7 +760,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -772,6 +775,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010011DB5BA7A27696418C6D2C8B46A68E83" ma:contentTypeVersion="17" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="b3e823de345af38b5a0fa8b2c9729ead">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="398d2b5b-77f8-4c5f-a794-3d35ce849315" xmlns:ns3="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7fae56da9623201e330c5b1623e145d1" ns2:_="" ns3:_="">
     <xsd:import namespace="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
@@ -1008,27 +1031,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46FCC551-4FF5-46A3-9024-D54BBA18C5A1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2633B21-6509-4402-A676-EEE1878D6EA1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
+    <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB9A7DEF-8D50-4222-A255-A8C989265833}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1045,23 +1067,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2633B21-6509-4402-A676-EEE1878D6EA1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
-    <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46FCC551-4FF5-46A3-9024-D54BBA18C5A1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Reconcile fixtures and tests with v6 schema after main merge
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Scenarios.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Scenarios.xlsx
@@ -1,27 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\pi-workflow\inst\extdata\examples\TestProject\Configurations\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E4FF0C-5C09-44C4-A351-7C0A443B5309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7460" yWindow="1190" windowWidth="27640" windowHeight="19270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7460" yWindow="1190" windowWidth="27640" windowHeight="19270" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Scenarios" sheetId="1" r:id="rId1"/>
-    <sheet name="OutputPaths" sheetId="2" r:id="rId2"/>
+    <sheet name="OutputPaths" sheetId="2" state="visible" r:id="rId1"/>
+    <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>Scenario_name</t>
   </si>
@@ -153,13 +146,134 @@
   </si>
   <si>
     <t>Organism|Fat|Intracellular|Aciclovir|Concentration in container</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IndividualId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PopulationId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ReadPopulationFromCSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ModelParameterSheets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ApplicationProtocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SimulationTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SimulationTimeUnit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SteadyState</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SteadyStateTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SteadyStateTimeUnit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OverwriteFormulasInSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ModelFile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OutputPathsIds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestScenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indiv1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aciclovir_iv_250mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0, 24, 60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aciclovir.pkml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aciclovir_PVB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestScenario2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Global", "Aciclovir", "Sheet, with comma"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0, 1, 60; 1, 12, 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aciclovir_PVB, Aciclovir_fat_cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PopulationScenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestPopulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0, 12, 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PopulationScenarioFromCSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TestScenario_missingParam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global, MissingParam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PITestScenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIScenario_250mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aciclovir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol_250mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,120,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIScenario_500mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol_500mg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,12 +282,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -196,13 +315,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -506,296 +624,346 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7265625" customWidth="1"/>
-    <col min="7" max="7" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>500</v>
-      </c>
-      <c r="K3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>18</v>
-      </c>
-      <c r="L6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>31</v>
-      </c>
-      <c r="L7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" t="b">
-        <v>0</v>
-      </c>
-      <c r="L8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" t="b">
-        <v>0</v>
-      </c>
-      <c r="L9" t="s">
-        <v>19</v>
+      <c r="B2" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>43</v>
-      </c>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M1" t="s">
+        <v>56</v>
+      </c>
+      <c r="N1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2"/>
+      <c r="L2"/>
+      <c r="M2" t="s">
+        <v>64</v>
+      </c>
+      <c r="N2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" t="s">
+        <v>63</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>500</v>
+      </c>
+      <c r="K3" t="s">
+        <v>69</v>
+      </c>
+      <c r="L3"/>
+      <c r="M3" t="s">
+        <v>64</v>
+      </c>
+      <c r="N3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4" t="s">
+        <v>64</v>
+      </c>
+      <c r="N4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5" t="s">
+        <v>63</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5" t="s">
+        <v>64</v>
+      </c>
+      <c r="N5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7" t="s">
+        <v>64</v>
+      </c>
+      <c r="N7"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8" t="s">
+        <v>64</v>
+      </c>
+      <c r="N8"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9" t="s">
+        <v>64</v>
+      </c>
+      <c r="N9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>